<commit_message>
Version 1.1.0: revision for Journal of Cheminformatics
Revised analysis code and outputs for the revision (October 2026) .
See CHANGELOG_revision.md and revision/README_revision.md.
</commit_message>
<xml_diff>
--- a/data/20260710_VIP_EffectSize_Tabellen.xlsx
+++ b/data/20260710_VIP_EffectSize_Tabellen.xlsx
@@ -18,6 +18,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VIP_Lit_S.Pyo" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VIP_ChemDes_P.A." sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VIP_Lit_P.A." sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FigS4c_axis_key" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,13 +28,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -56,8 +60,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,7 +483,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Route B uses 12 of the 25 literature descriptors (unsupervised correlation reduction; one further pair is exactly redundant and reduces to a single representative, see Table S4); empty RouteB cells = removed in the correlation step.</t>
+          <t>Route B uses 12 of the 25 literature descriptors (unsupervised correlation reduction; one further pair is exactly redundant and reduces to a single representative, see Table S7); empty RouteB cells = removed in the correlation step.</t>
         </is>
       </c>
     </row>
@@ -486,6 +491,21 @@
       <c r="A9" t="inlineStr">
         <is>
           <t>Note: VIP here is from two components (as in MetaboAnalyst); the validated Q² models used one component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>FigS4c_axis_key: the Fig. S4c x-axis is numbered 1-60 (union of the five strain-specific Route A1 top-15 sets, ordered by mean VIP); this sheet gives the descriptor name for each position number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>REVISION (03.10.2026): in the VIP_Lit sheets the columns TwoStage_VIP_apparent, TwoStage_VIP_nested_mean, TwoStage_selfreq_VIPgt1 and EffectSize, which use all 25 literature descriptors, were recomputed with the corrected stereocentre count of 1,8-cineole (0 instead of 2; see the Route B descriptor file). Rows are again sorted by TwoStage_VIP_apparent. The RouteB columns (12-descriptor set, which does not contain NumStereoCenters) and the ChemDes sheets are unchanged. The EffectSize of MolWt is now computed with ties between isomers of the same formula, which the submitted values had broken because of floating-point noise in the 14th decimal (change at most 0.024).</t>
         </is>
       </c>
     </row>
@@ -909,10 +929,10 @@
         <v>2.402</v>
       </c>
       <c r="D2" t="n">
-        <v>2.883</v>
+        <v>2.898</v>
       </c>
       <c r="E2" t="n">
-        <v>2.879</v>
+        <v>2.894</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -936,10 +956,10 @@
         <v>1.807</v>
       </c>
       <c r="D3" t="n">
-        <v>2.115</v>
+        <v>2.129</v>
       </c>
       <c r="E3" t="n">
-        <v>2.109</v>
+        <v>2.123</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -953,7 +973,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FractionCSP3</t>
+          <t>NumHDonors</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -963,10 +983,10 @@
         <v>1.178</v>
       </c>
       <c r="D4" t="n">
-        <v>1.344</v>
+        <v>1.353</v>
       </c>
       <c r="E4" t="n">
-        <v>1.339</v>
+        <v>1.349</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -974,28 +994,34 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>0.905</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NumHDonors</t>
-        </is>
+          <t>FractionCSP3</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1.181</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1.178</v>
       </c>
       <c r="D5" t="n">
+        <v>1.349</v>
+      </c>
+      <c r="E5" t="n">
         <v>1.344</v>
       </c>
-      <c r="E5" t="n">
-        <v>1.34</v>
-      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>31/31</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>0.75</v>
+        <v>0.905</v>
       </c>
     </row>
     <row r="6">
@@ -1005,10 +1031,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1.185</v>
+        <v>1.192</v>
       </c>
       <c r="E6" t="n">
-        <v>1.181</v>
+        <v>1.188</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1022,18 +1048,18 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NumStereoCenters</t>
+          <t>NumAliphaticRings</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.043</v>
+        <v>1.007</v>
       </c>
       <c r="E7" t="n">
-        <v>1.04</v>
+        <v>1.004</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>28/31</t>
+          <t>20/31</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -1043,22 +1069,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NumAliphaticRings</t>
+          <t>NumStereoCenters</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1.014</v>
+        <v>0.97</v>
       </c>
       <c r="E8" t="n">
-        <v>1.01</v>
+        <v>0.968</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>22/31</t>
+          <t>7/31</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>0.679</v>
+        <v>0.643</v>
       </c>
     </row>
     <row r="9">
@@ -1074,10 +1100,10 @@
         <v>0.7</v>
       </c>
       <c r="D9" t="n">
-        <v>0.88</v>
+        <v>0.878</v>
       </c>
       <c r="E9" t="n">
-        <v>0.878</v>
+        <v>0.875</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1101,10 +1127,10 @@
         <v>0.644</v>
       </c>
       <c r="D10" t="n">
-        <v>0.783</v>
+        <v>0.787</v>
       </c>
       <c r="E10" t="n">
-        <v>0.782</v>
+        <v>0.785</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1122,10 +1148,10 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.722</v>
+        <v>0.73</v>
       </c>
       <c r="E11" t="n">
-        <v>0.727</v>
+        <v>0.735</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -1143,10 +1169,10 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.628</v>
+        <v>0.635</v>
       </c>
       <c r="E12" t="n">
-        <v>0.63</v>
+        <v>0.636</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -1170,10 +1196,10 @@
         <v>0.27</v>
       </c>
       <c r="D13" t="n">
-        <v>0.584</v>
+        <v>0.578</v>
       </c>
       <c r="E13" t="n">
-        <v>0.576</v>
+        <v>0.571</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -1187,14 +1213,14 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>NumRotatableBonds</t>
+          <t>HeavyAtomCount</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.577</v>
+        <v>0.573</v>
       </c>
       <c r="E14" t="n">
-        <v>0.576</v>
+        <v>0.575</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1202,20 +1228,20 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>0.143</v>
+        <v>0.333</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>HeavyAtomCount</t>
+          <t>NumRotatableBonds</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.5669999999999999</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="E15" t="n">
-        <v>0.57</v>
+        <v>0.5629999999999999</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1223,7 +1249,7 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>0.333</v>
+        <v>0.143</v>
       </c>
     </row>
     <row r="16">
@@ -1239,10 +1265,10 @@
         <v>0.415</v>
       </c>
       <c r="D16" t="n">
-        <v>0.524</v>
+        <v>0.525</v>
       </c>
       <c r="E16" t="n">
-        <v>0.526</v>
+        <v>0.527</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1260,10 +1286,10 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.464</v>
+        <v>0.471</v>
       </c>
       <c r="E17" t="n">
-        <v>0.478</v>
+        <v>0.484</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1277,7 +1303,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>RingCount</t>
+          <t>MolMR</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1287,10 +1313,10 @@
         <v>0.201</v>
       </c>
       <c r="D18" t="n">
-        <v>0.463</v>
+        <v>0.436</v>
       </c>
       <c r="E18" t="n">
-        <v>0.461</v>
+        <v>0.43</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1298,20 +1324,26 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MolMR</t>
-        </is>
+          <t>Aldehyde_flag</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.337</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.337</v>
       </c>
       <c r="D19" t="n">
-        <v>0.445</v>
+        <v>0.433</v>
       </c>
       <c r="E19" t="n">
-        <v>0.439</v>
+        <v>0.432</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1319,26 +1351,26 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>0.31</v>
+        <v>0.179</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Aldehyde_flag</t>
+          <t>RingCount</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.337</v>
+        <v>0.204</v>
       </c>
       <c r="C20" t="n">
-        <v>0.337</v>
+        <v>0.201</v>
       </c>
       <c r="D20" t="n">
-        <v>0.436</v>
+        <v>0.422</v>
       </c>
       <c r="E20" t="n">
-        <v>0.435</v>
+        <v>0.421</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1346,7 +1378,7 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>0.179</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -1356,10 +1388,10 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.408</v>
+        <v>0.414</v>
       </c>
       <c r="E21" t="n">
-        <v>0.418</v>
+        <v>0.424</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1367,7 +1399,7 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>0.06</v>
+        <v>0.036</v>
       </c>
     </row>
     <row r="22">
@@ -1383,10 +1415,10 @@
         <v>0.394</v>
       </c>
       <c r="D22" t="n">
-        <v>0.407</v>
+        <v>0.409</v>
       </c>
       <c r="E22" t="n">
-        <v>0.407</v>
+        <v>0.409</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1404,10 +1436,10 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.381</v>
+        <v>0.385</v>
       </c>
       <c r="E23" t="n">
-        <v>0.392</v>
+        <v>0.396</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1431,10 +1463,10 @@
         <v>0.294</v>
       </c>
       <c r="D24" t="n">
-        <v>0.335</v>
+        <v>0.302</v>
       </c>
       <c r="E24" t="n">
-        <v>0.333</v>
+        <v>0.3</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1452,10 +1484,10 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.228</v>
+        <v>0.226</v>
       </c>
       <c r="E25" t="n">
-        <v>0.226</v>
+        <v>0.224</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1479,10 +1511,10 @@
         <v>0.14</v>
       </c>
       <c r="D26" t="n">
-        <v>0.228</v>
+        <v>0.226</v>
       </c>
       <c r="E26" t="n">
-        <v>0.226</v>
+        <v>0.224</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1491,6 +1523,636 @@
       </c>
       <c r="G26" t="n">
         <v>0.036</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B61"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Descriptor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>BlueDesc_mmff94::count.AromaticOHGroups</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Chemopy_1D2D::EstateVSA6</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PaDEL_3D::RDF55s</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PaDEL_1D2D::ETA_Eta_F_L</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PaDEL_3D::TDB4s</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Chemopy_1D2D::EstateVSA9</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>PaDEL_1D2D::maxHother</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PaDEL_1D2D::SpMin8_Bhs</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>PaDEL_1D2D::SM1_Dzs</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Chemopy_3D::MoRSEC22</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PaDEL_1D2D::minwHBa</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Chemopy_1D2D::CIC2</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PaDEL_3D::E3e</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>PaDEL_3D::TDB5e</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Chemopy_1D2D::SIC1</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Chemopy_3D::MoRSEV28</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Chemopy_3D::MoRSEU18</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>PaDEL_3D::Vv</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>PaDEL_1D2D::MATS3e</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>PaDEL_3D::FPSA-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Chemopy_3D::MoRSEE28</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Chemopy_3D::MoRSEE29</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Chemopy_3D::MoRSEU29</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>BlueDesc_mmff94::RPCS</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>PaDEL_3D::TDB3r</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>BlueDesc_mmff94::FPSA-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Chemopy_3D::MoRSEM18</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Chemopy_3D::RDFM9</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>PaDEL_3D::TDB5v</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Chemopy_3D::MoRSEU11</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Chemopy_1D2D::ATSv4</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>PaDEL_3D::RDF40u</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>PaDEL_3D::E3i</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>PaDEL_1D2D::AATSC3v</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>PaDEL_1D2D::hmin</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>PaDEL_1D2D::AVP-7</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Chemopy_3D::Te</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Chemopy_1D2D::Qmin</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Chemopy_1D2D::Smin8</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>PaDEL_3D::THSA</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>PaDEL_1D2D::AATS5m</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>PaDEL_1D2D::AATSC8s</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Chemopy_3D::MoRSEM8</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Chemopy_3D::RDFU7</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>BlueDesc_mmff94::SCH-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Chemopy_3D::E3m</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>PaDEL_3D::RDF55m</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>PaDEL_3D::Du</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>PaDEL_1D2D::SpMin4_Bhs</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>PaDEL_3D::RDF35i</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>PaDEL_1D2D::SpMin7_Bhs</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>PaDEL_1D2D::AATSC1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>PaDEL_1D2D::AATSC8v</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>PaDEL_3D::GRAVH-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>PaDEL_1D2D::MATS1e</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Chemopy_3D::MoRSEE27</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Chemopy_3D::RDFU6</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>PaDEL_3D::RDF40p</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>PaDEL_1D2D::AATSC8m</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>PaDEL_3D::MOMI-XY</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1913,10 +2575,10 @@
         <v>1.405</v>
       </c>
       <c r="D2" t="n">
-        <v>1.645</v>
+        <v>1.647</v>
       </c>
       <c r="E2" t="n">
-        <v>1.638</v>
+        <v>1.641</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1940,10 +2602,10 @@
         <v>1.378</v>
       </c>
       <c r="D3" t="n">
-        <v>1.517</v>
+        <v>1.53</v>
       </c>
       <c r="E3" t="n">
-        <v>1.511</v>
+        <v>1.524</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1967,10 +2629,10 @@
         <v>1.456</v>
       </c>
       <c r="D4" t="n">
-        <v>1.477</v>
+        <v>1.495</v>
       </c>
       <c r="E4" t="n">
-        <v>1.472</v>
+        <v>1.491</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1994,10 +2656,10 @@
         <v>0.844</v>
       </c>
       <c r="D5" t="n">
-        <v>1.358</v>
+        <v>1.34</v>
       </c>
       <c r="E5" t="n">
-        <v>1.347</v>
+        <v>1.33</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -2015,10 +2677,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1.275</v>
+        <v>1.282</v>
       </c>
       <c r="E6" t="n">
-        <v>1.271</v>
+        <v>1.278</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -2032,76 +2694,82 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NumStereoCenters</t>
+          <t>NumHAcceptors</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.109</v>
+        <v>1.111</v>
       </c>
       <c r="E7" t="n">
-        <v>1.11</v>
+        <v>1.105</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>30/31</t>
+          <t>29/31</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>0.41</v>
+        <v>0.371</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NumHAcceptors</t>
-        </is>
+          <t>RingCount</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1.026</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1.023</v>
       </c>
       <c r="D8" t="n">
-        <v>1.094</v>
+        <v>1.056</v>
       </c>
       <c r="E8" t="n">
-        <v>1.089</v>
+        <v>1.053</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>29/31</t>
+          <t>25/31</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>0.371</v>
+        <v>0.343</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>RingCount</t>
+          <t>TPSA</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1.026</v>
+        <v>1.104</v>
       </c>
       <c r="C9" t="n">
-        <v>1.023</v>
+        <v>1.101</v>
       </c>
       <c r="D9" t="n">
-        <v>1.055</v>
+        <v>1.042</v>
       </c>
       <c r="E9" t="n">
-        <v>1.052</v>
+        <v>1.037</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>25/31</t>
+          <t>21/31</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>0.343</v>
+        <v>0.452</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TPSA</t>
+          <t>DegreeUnsaturation</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -2111,60 +2779,60 @@
         <v>1.101</v>
       </c>
       <c r="D10" t="n">
-        <v>1.024</v>
+        <v>1.017</v>
       </c>
       <c r="E10" t="n">
-        <v>1.02</v>
+        <v>1.014</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>20/31</t>
+          <t>17/31</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>0.452</v>
+        <v>0.376</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DegreeUnsaturation</t>
+          <t>MolMR</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1.005</v>
+        <v>0.963</v>
       </c>
       <c r="E11" t="n">
-        <v>1.002</v>
+        <v>0.959</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>17/31</t>
+          <t>9/31</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>0.376</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MolMR</t>
+          <t>NumStereoCenters</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.958</v>
+        <v>0.96</v>
       </c>
       <c r="E12" t="n">
-        <v>0.955</v>
+        <v>0.961</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>8/31</t>
+          <t>9/31</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>0.39</v>
+        <v>0.352</v>
       </c>
     </row>
     <row r="13">
@@ -2174,10 +2842,10 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.911</v>
+        <v>0.913</v>
       </c>
       <c r="E13" t="n">
-        <v>0.911</v>
+        <v>0.912</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -2195,14 +2863,14 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.886</v>
+        <v>0.906</v>
       </c>
       <c r="E14" t="n">
-        <v>0.881</v>
+        <v>0.901</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1/31</t>
+          <t>2/31</t>
         </is>
       </c>
       <c r="G14" t="n">
@@ -2216,14 +2884,14 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.844</v>
+        <v>0.857</v>
       </c>
       <c r="E15" t="n">
-        <v>0.843</v>
+        <v>0.856</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0/31</t>
+          <t>2/31</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -2237,14 +2905,14 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.832</v>
+        <v>0.85</v>
       </c>
       <c r="E16" t="n">
-        <v>0.828</v>
+        <v>0.845</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1/31</t>
+          <t>2/31</t>
         </is>
       </c>
       <c r="G16" t="n">
@@ -2264,10 +2932,10 @@
         <v>0.968</v>
       </c>
       <c r="D17" t="n">
-        <v>0.819</v>
+        <v>0.829</v>
       </c>
       <c r="E17" t="n">
-        <v>0.8169999999999999</v>
+        <v>0.827</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -2281,14 +2949,14 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>LabuteASA</t>
+          <t>MolWt</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.748</v>
+        <v>0.764</v>
       </c>
       <c r="E18" t="n">
-        <v>0.743</v>
+        <v>0.758</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -2296,20 +2964,20 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>0.171</v>
+        <v>0.119</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MolWt</t>
+          <t>LabuteASA</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.746</v>
+        <v>0.763</v>
       </c>
       <c r="E19" t="n">
-        <v>0.741</v>
+        <v>0.758</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -2317,34 +2985,34 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>0.133</v>
+        <v>0.171</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>EsterLacton_flag</t>
+          <t>Ketone_flag</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.441</v>
+        <v>0.726</v>
       </c>
       <c r="C20" t="n">
-        <v>0.433</v>
+        <v>0.725</v>
       </c>
       <c r="D20" t="n">
+        <v>0.727</v>
+      </c>
+      <c r="E20" t="n">
         <v>0.728</v>
       </c>
-      <c r="E20" t="n">
-        <v>0.709</v>
-      </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0/31</t>
+          <t>1/31</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>0.048</v>
+        <v>0.186</v>
       </c>
     </row>
     <row r="21">
@@ -2354,10 +3022,10 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.728</v>
+        <v>0.717</v>
       </c>
       <c r="E21" t="n">
-        <v>0.709</v>
+        <v>0.699</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -2371,28 +3039,28 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Ketone_flag</t>
+          <t>EsterLacton_flag</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.726</v>
+        <v>0.441</v>
       </c>
       <c r="C22" t="n">
-        <v>0.725</v>
+        <v>0.433</v>
       </c>
       <c r="D22" t="n">
-        <v>0.725</v>
+        <v>0.717</v>
       </c>
       <c r="E22" t="n">
-        <v>0.726</v>
+        <v>0.699</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>1/31</t>
+          <t>0/31</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>0.186</v>
+        <v>0.048</v>
       </c>
     </row>
     <row r="23">
@@ -2408,10 +3076,10 @@
         <v>0.579</v>
       </c>
       <c r="D23" t="n">
-        <v>0.6909999999999999</v>
+        <v>0.703</v>
       </c>
       <c r="E23" t="n">
-        <v>0.6909999999999999</v>
+        <v>0.703</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -2429,10 +3097,10 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.68</v>
       </c>
       <c r="E24" t="n">
-        <v>0.6929999999999999</v>
+        <v>0.6830000000000001</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -2456,7 +3124,7 @@
         <v>0.65</v>
       </c>
       <c r="D25" t="n">
-        <v>0.574</v>
+        <v>0.575</v>
       </c>
       <c r="E25" t="n">
         <v>0.575</v>
@@ -2483,10 +3151,10 @@
         <v>0.745</v>
       </c>
       <c r="D26" t="n">
-        <v>0.389</v>
+        <v>0.381</v>
       </c>
       <c r="E26" t="n">
-        <v>0.403</v>
+        <v>0.396</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -2917,10 +3585,10 @@
         <v>2.063</v>
       </c>
       <c r="D2" t="n">
-        <v>2.32</v>
+        <v>2.331</v>
       </c>
       <c r="E2" t="n">
-        <v>2.312</v>
+        <v>2.323</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2944,10 +3612,10 @@
         <v>1.532</v>
       </c>
       <c r="D3" t="n">
-        <v>1.684</v>
+        <v>1.698</v>
       </c>
       <c r="E3" t="n">
-        <v>1.679</v>
+        <v>1.693</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2971,10 +3639,10 @@
         <v>1.543</v>
       </c>
       <c r="D4" t="n">
-        <v>1.589</v>
+        <v>1.601</v>
       </c>
       <c r="E4" t="n">
-        <v>1.582</v>
+        <v>1.593</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -2992,10 +3660,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1.533</v>
+        <v>1.545</v>
       </c>
       <c r="E5" t="n">
-        <v>1.528</v>
+        <v>1.539</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -3013,10 +3681,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1.418</v>
+        <v>1.342</v>
       </c>
       <c r="E6" t="n">
-        <v>1.415</v>
+        <v>1.339</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -3024,7 +3692,7 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>0.731</v>
+        <v>0.6919999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -3034,10 +3702,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.128</v>
+        <v>1.14</v>
       </c>
       <c r="E7" t="n">
-        <v>1.123</v>
+        <v>1.134</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -3055,14 +3723,14 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1.082</v>
+        <v>1.081</v>
       </c>
       <c r="E8" t="n">
-        <v>1.08</v>
+        <v>1.079</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>28/31</t>
+          <t>27/31</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -3082,14 +3750,14 @@
         <v>1.102</v>
       </c>
       <c r="D9" t="n">
-        <v>1.035</v>
+        <v>1.045</v>
       </c>
       <c r="E9" t="n">
-        <v>1.031</v>
+        <v>1.04</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>26/31</t>
+          <t>27/31</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -3099,7 +3767,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CarboxAcid_flag</t>
+          <t>O_Count</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -3109,10 +3777,10 @@
         <v>0.705</v>
       </c>
       <c r="D10" t="n">
-        <v>0.919</v>
+        <v>0.931</v>
       </c>
       <c r="E10" t="n">
-        <v>0.916</v>
+        <v>0.926</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -3120,28 +3788,34 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>0.077</v>
+        <v>0.431</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>O_Count</t>
-        </is>
+          <t>CarboxAcid_flag</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.716</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.705</v>
       </c>
       <c r="D11" t="n">
-        <v>0.918</v>
+        <v>0.911</v>
       </c>
       <c r="E11" t="n">
-        <v>0.913</v>
+        <v>0.908</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>4/31</t>
+          <t>2/31</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>0.431</v>
+        <v>0.077</v>
       </c>
     </row>
     <row r="12">
@@ -3151,10 +3825,10 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.843</v>
+        <v>0.85</v>
       </c>
       <c r="E12" t="n">
-        <v>0.839</v>
+        <v>0.846</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -3172,14 +3846,14 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.833</v>
+        <v>0.845</v>
       </c>
       <c r="E13" t="n">
-        <v>0.828</v>
+        <v>0.84</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1/31</t>
+          <t>2/31</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -3193,10 +3867,10 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.805</v>
+        <v>0.8110000000000001</v>
       </c>
       <c r="E14" t="n">
-        <v>0.802</v>
+        <v>0.8080000000000001</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -3214,10 +3888,10 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.634</v>
+        <v>0.646</v>
       </c>
       <c r="E15" t="n">
-        <v>0.63</v>
+        <v>0.642</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -3225,7 +3899,7 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>0.123</v>
+        <v>0.131</v>
       </c>
     </row>
     <row r="16">
@@ -3235,10 +3909,10 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.626</v>
+        <v>0.62</v>
       </c>
       <c r="E16" t="n">
-        <v>0.627</v>
+        <v>0.62</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -3256,10 +3930,10 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.593</v>
+        <v>0.604</v>
       </c>
       <c r="E17" t="n">
-        <v>0.59</v>
+        <v>0.601</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -3283,10 +3957,10 @@
         <v>0.578</v>
       </c>
       <c r="D18" t="n">
-        <v>0.586</v>
+        <v>0.589</v>
       </c>
       <c r="E18" t="n">
-        <v>0.586</v>
+        <v>0.589</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -3310,10 +3984,10 @@
         <v>0.466</v>
       </c>
       <c r="D19" t="n">
-        <v>0.575</v>
+        <v>0.549</v>
       </c>
       <c r="E19" t="n">
-        <v>0.578</v>
+        <v>0.552</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -3327,7 +4001,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>EsterLacton_flag</t>
+          <t>C_Count</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -3337,10 +4011,10 @@
         <v>0.259</v>
       </c>
       <c r="D20" t="n">
-        <v>0.458</v>
+        <v>0.453</v>
       </c>
       <c r="E20" t="n">
-        <v>0.449</v>
+        <v>0.444</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -3354,14 +4028,20 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>C_Count</t>
-        </is>
+          <t>EsterLacton_flag</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.264</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.259</v>
       </c>
       <c r="D21" t="n">
-        <v>0.458</v>
+        <v>0.453</v>
       </c>
       <c r="E21" t="n">
-        <v>0.449</v>
+        <v>0.444</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -3379,10 +4059,10 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.458</v>
+        <v>0.434</v>
       </c>
       <c r="E22" t="n">
-        <v>0.463</v>
+        <v>0.439</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -3406,10 +4086,10 @@
         <v>0.504</v>
       </c>
       <c r="D23" t="n">
-        <v>0.399</v>
+        <v>0.374</v>
       </c>
       <c r="E23" t="n">
-        <v>0.399</v>
+        <v>0.373</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -3433,10 +4113,10 @@
         <v>0.196</v>
       </c>
       <c r="D24" t="n">
-        <v>0.146</v>
+        <v>0.144</v>
       </c>
       <c r="E24" t="n">
-        <v>0.182</v>
+        <v>0.181</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -3487,10 +4167,10 @@
         <v>0.228</v>
       </c>
       <c r="D26" t="n">
-        <v>0.058</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="E26" t="n">
-        <v>0.111</v>
+        <v>0.119</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -3921,10 +4601,10 @@
         <v>1.864</v>
       </c>
       <c r="D2" t="n">
-        <v>2.086</v>
+        <v>2.102</v>
       </c>
       <c r="E2" t="n">
-        <v>2.078</v>
+        <v>2.093</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3948,10 +4628,10 @@
         <v>1.629</v>
       </c>
       <c r="D3" t="n">
-        <v>1.792</v>
+        <v>1.811</v>
       </c>
       <c r="E3" t="n">
-        <v>1.786</v>
+        <v>1.804</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3969,10 +4649,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1.691</v>
+        <v>1.707</v>
       </c>
       <c r="E4" t="n">
-        <v>1.684</v>
+        <v>1.7</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -3990,10 +4670,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1.606</v>
+        <v>1.524</v>
       </c>
       <c r="E5" t="n">
-        <v>1.601</v>
+        <v>1.519</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -4001,7 +4681,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>0.76</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="6">
@@ -4017,10 +4697,10 @@
         <v>1.385</v>
       </c>
       <c r="D6" t="n">
-        <v>1.385</v>
+        <v>1.399</v>
       </c>
       <c r="E6" t="n">
-        <v>1.378</v>
+        <v>1.392</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -4038,10 +4718,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.102</v>
+        <v>1.115</v>
       </c>
       <c r="E7" t="n">
-        <v>1.098</v>
+        <v>1.11</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -4059,10 +4739,10 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1.033</v>
+        <v>1.026</v>
       </c>
       <c r="E8" t="n">
-        <v>1.031</v>
+        <v>1.024</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -4086,14 +4766,14 @@
         <v>1.105</v>
       </c>
       <c r="D9" t="n">
-        <v>0.976</v>
+        <v>0.988</v>
       </c>
       <c r="E9" t="n">
-        <v>0.971</v>
+        <v>0.982</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>8/31</t>
+          <t>9/31</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -4113,10 +4793,10 @@
         <v>0.722</v>
       </c>
       <c r="D10" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="E10" t="n">
-        <v>0.9389999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -4134,14 +4814,14 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.914</v>
+        <v>0.921</v>
       </c>
       <c r="E11" t="n">
-        <v>0.913</v>
+        <v>0.92</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>4/31</t>
+          <t>5/31</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -4155,10 +4835,10 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.868</v>
+        <v>0.883</v>
       </c>
       <c r="E12" t="n">
-        <v>0.862</v>
+        <v>0.878</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -4176,10 +4856,10 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.777</v>
+        <v>0.792</v>
       </c>
       <c r="E13" t="n">
-        <v>0.772</v>
+        <v>0.787</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -4203,14 +4883,14 @@
         <v>0.759</v>
       </c>
       <c r="D14" t="n">
-        <v>0.753</v>
+        <v>0.761</v>
       </c>
       <c r="E14" t="n">
-        <v>0.753</v>
+        <v>0.76</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0/31</t>
+          <t>1/31</t>
         </is>
       </c>
       <c r="G14" t="n">
@@ -4230,10 +4910,10 @@
         <v>0.651</v>
       </c>
       <c r="D15" t="n">
-        <v>0.66</v>
+        <v>0.667</v>
       </c>
       <c r="E15" t="n">
-        <v>0.66</v>
+        <v>0.668</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -4251,10 +4931,10 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.602</v>
+        <v>0.606</v>
       </c>
       <c r="E16" t="n">
-        <v>0.6</v>
+        <v>0.605</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -4272,10 +4952,10 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.601</v>
+        <v>0.59</v>
       </c>
       <c r="E17" t="n">
-        <v>0.601</v>
+        <v>0.591</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4289,7 +4969,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>RingCount</t>
+          <t>MolWt</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4299,10 +4979,10 @@
         <v>0.61</v>
       </c>
       <c r="D18" t="n">
-        <v>0.6</v>
+        <v>0.571</v>
       </c>
       <c r="E18" t="n">
-        <v>0.602</v>
+        <v>0.5659999999999999</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4310,20 +4990,26 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>0.16</v>
+        <v>0.027</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>NumRotatableBonds</t>
-        </is>
+          <t>RingCount</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.611</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.61</v>
       </c>
       <c r="D19" t="n">
         <v>0.5659999999999999</v>
       </c>
       <c r="E19" t="n">
-        <v>0.571</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4331,20 +5017,20 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MolWt</t>
+          <t>NumRotatableBonds</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.5570000000000001</v>
+        <v>0.539</v>
       </c>
       <c r="E20" t="n">
-        <v>0.552</v>
+        <v>0.544</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4352,7 +5038,7 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>0.013</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -4362,10 +5048,10 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.524</v>
+        <v>0.536</v>
       </c>
       <c r="E21" t="n">
-        <v>0.521</v>
+        <v>0.533</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -4383,10 +5069,10 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.474</v>
+        <v>0.468</v>
       </c>
       <c r="E22" t="n">
-        <v>0.464</v>
+        <v>0.459</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -4410,10 +5096,10 @@
         <v>0.298</v>
       </c>
       <c r="D23" t="n">
-        <v>0.474</v>
+        <v>0.468</v>
       </c>
       <c r="E23" t="n">
-        <v>0.464</v>
+        <v>0.459</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -4437,10 +5123,10 @@
         <v>0.524</v>
       </c>
       <c r="D24" t="n">
-        <v>0.439</v>
+        <v>0.414</v>
       </c>
       <c r="E24" t="n">
-        <v>0.439</v>
+        <v>0.413</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -4464,10 +5150,10 @@
         <v>0.307</v>
       </c>
       <c r="D25" t="n">
-        <v>0.286</v>
+        <v>0.299</v>
       </c>
       <c r="E25" t="n">
-        <v>0.296</v>
+        <v>0.308</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -4925,10 +5611,10 @@
         <v>1.55</v>
       </c>
       <c r="D2" t="n">
-        <v>1.544</v>
+        <v>1.548</v>
       </c>
       <c r="E2" t="n">
-        <v>1.534</v>
+        <v>1.538</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4949,7 +5635,7 @@
         <v>1.537</v>
       </c>
       <c r="E3" t="n">
-        <v>1.529</v>
+        <v>1.528</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4997,7 +5683,7 @@
         <v>1.437</v>
       </c>
       <c r="E5" t="n">
-        <v>1.43</v>
+        <v>1.431</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -5015,10 +5701,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1.42</v>
+        <v>1.421</v>
       </c>
       <c r="E6" t="n">
-        <v>1.413</v>
+        <v>1.415</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -5026,7 +5712,7 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.582</v>
       </c>
     </row>
     <row r="7">
@@ -5036,10 +5722,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.412</v>
+        <v>1.414</v>
       </c>
       <c r="E7" t="n">
-        <v>1.406</v>
+        <v>1.407</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -5057,10 +5743,10 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1.411</v>
+        <v>1.412</v>
       </c>
       <c r="E8" t="n">
-        <v>1.405</v>
+        <v>1.406</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -5078,10 +5764,10 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1.262</v>
+        <v>1.261</v>
       </c>
       <c r="E9" t="n">
-        <v>1.256</v>
+        <v>1.255</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -5099,14 +5785,14 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1.076</v>
+        <v>1.086</v>
       </c>
       <c r="E10" t="n">
-        <v>1.07</v>
+        <v>1.08</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>27/31</t>
+          <t>28/31</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -5126,10 +5812,10 @@
         <v>0.713</v>
       </c>
       <c r="D11" t="n">
-        <v>1.023</v>
+        <v>1.02</v>
       </c>
       <c r="E11" t="n">
-        <v>1.035</v>
+        <v>1.033</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -5143,28 +5829,34 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>NumHDonors</t>
-        </is>
+          <t>NumAromaticRings</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1.004</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.991</v>
       </c>
       <c r="D12" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.947</v>
       </c>
       <c r="E12" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>9/31</t>
+          <t>6/31</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>0.345</v>
+        <v>0.173</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>NumAromaticRings</t>
+          <t>NumHDonors</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -5174,18 +5866,18 @@
         <v>0.991</v>
       </c>
       <c r="D13" t="n">
-        <v>0.9360000000000001</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="E13" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>5/31</t>
+          <t>9/31</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>0.173</v>
+        <v>0.345</v>
       </c>
     </row>
     <row r="14">
@@ -5201,10 +5893,10 @@
         <v>0.848</v>
       </c>
       <c r="D14" t="n">
-        <v>0.879</v>
+        <v>0.866</v>
       </c>
       <c r="E14" t="n">
-        <v>0.877</v>
+        <v>0.864</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -5222,10 +5914,10 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.849</v>
+        <v>0.852</v>
       </c>
       <c r="E15" t="n">
-        <v>0.848</v>
+        <v>0.852</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -5249,10 +5941,10 @@
         <v>1.117</v>
       </c>
       <c r="D16" t="n">
-        <v>0.839</v>
+        <v>0.843</v>
       </c>
       <c r="E16" t="n">
-        <v>0.837</v>
+        <v>0.84</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -5270,10 +5962,10 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.769</v>
+        <v>0.767</v>
       </c>
       <c r="E17" t="n">
-        <v>0.773</v>
+        <v>0.77</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -5297,10 +5989,10 @@
         <v>0.752</v>
       </c>
       <c r="D18" t="n">
-        <v>0.665</v>
+        <v>0.677</v>
       </c>
       <c r="E18" t="n">
-        <v>0.662</v>
+        <v>0.673</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -5314,7 +6006,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>EsterLacton_flag</t>
+          <t>C_Count</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -5341,8 +6033,14 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>C_Count</t>
-        </is>
+          <t>EsterLacton_flag</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.988</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.965</v>
       </c>
       <c r="D20" t="n">
         <v>0.654</v>
@@ -5362,14 +6060,20 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>NumStereoCenters</t>
-        </is>
+          <t>FractionCSP3</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.757</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.748</v>
       </c>
       <c r="D21" t="n">
-        <v>0.383</v>
+        <v>0.364</v>
       </c>
       <c r="E21" t="n">
-        <v>0.385</v>
+        <v>0.366</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -5377,26 +6081,26 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>0.159</v>
+        <v>0.136</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>FractionCSP3</t>
+          <t>Alcohol_flag</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.757</v>
+        <v>0.168</v>
       </c>
       <c r="C22" t="n">
-        <v>0.748</v>
+        <v>0.203</v>
       </c>
       <c r="D22" t="n">
-        <v>0.348</v>
+        <v>0.301</v>
       </c>
       <c r="E22" t="n">
-        <v>0.351</v>
+        <v>0.324</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -5404,13 +6108,13 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>0.136</v>
+        <v>0.032</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Alcohol_flag</t>
+          <t>NumStereoCenters</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -5420,10 +6124,10 @@
         <v>0.203</v>
       </c>
       <c r="D23" t="n">
-        <v>0.294</v>
+        <v>0.256</v>
       </c>
       <c r="E23" t="n">
-        <v>0.317</v>
+        <v>0.26</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -5431,26 +6135,26 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>0.032</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ketone_flag</t>
+          <t>Aldehyde_flag</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.332</v>
+        <v>0.405</v>
       </c>
       <c r="C24" t="n">
-        <v>0.342</v>
+        <v>0.422</v>
       </c>
       <c r="D24" t="n">
-        <v>0.22</v>
+        <v>0.222</v>
       </c>
       <c r="E24" t="n">
-        <v>0.243</v>
+        <v>0.252</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -5458,23 +6162,23 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>0.073</v>
+        <v>0.032</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Aldehyde_flag</t>
+          <t>Ketone_flag</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.405</v>
+        <v>0.332</v>
       </c>
       <c r="C25" t="n">
-        <v>0.422</v>
+        <v>0.342</v>
       </c>
       <c r="D25" t="n">
-        <v>0.213</v>
+        <v>0.221</v>
       </c>
       <c r="E25" t="n">
         <v>0.244</v>
@@ -5485,7 +6189,7 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>0.032</v>
+        <v>0.073</v>
       </c>
     </row>
     <row r="26">
@@ -5495,10 +6199,10 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.068</v>
+        <v>0.075</v>
       </c>
       <c r="E26" t="n">
-        <v>0.121</v>
+        <v>0.124</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>

</xml_diff>